<commit_message>
fix: JS leak in Product Create, clean debug logs, print invoice styling, hero stats center, admin logo, dashboard products count fix, Categories Create redesign
</commit_message>
<xml_diff>
--- a/Orkideya/wwwroot/orders.xlsx
+++ b/Orkideya/wwwroot/orders.xlsx
@@ -243,6 +243,39 @@
   </x:si>
   <x:si>
     <x:t>زيت السمسم (50)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>كككك</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-02-25 05:05</x:t>
+  </x:si>
+  <x:si>
+    <x:t>مؤيد فؤاد  بغني</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">عين زاره </x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-02-25 06:25</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Mohannd Fouad</x:t>
+  </x:si>
+  <x:si>
+    <x:t>0911189892</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-02-25 19:55</x:t>
+  </x:si>
+  <x:si>
+    <x:t>فانوس رمضان</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ليبيا</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-02-26 03:46</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -1847,6 +1880,180 @@
         <x:v>105</x:v>
       </x:c>
     </x:row>
+    <x:row r="44" spans="1:9">
+      <x:c r="A44" s="0">
+        <x:v>1027</x:v>
+      </x:c>
+      <x:c r="B44" s="0" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="C44" s="0" t="s">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="D44" s="0" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="E44" s="0" t="s">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="F44" s="0" t="s">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="G44" s="0" t="s">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="H44" s="0">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I44" s="0">
+        <x:v>100</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" spans="1:9">
+      <x:c r="A45" s="0">
+        <x:v>1028</x:v>
+      </x:c>
+      <x:c r="B45" s="0" t="s">
+        <x:v>76</x:v>
+      </x:c>
+      <x:c r="C45" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="D45" s="0" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="E45" s="0" t="s">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="F45" s="0" t="s">
+        <x:v>78</x:v>
+      </x:c>
+      <x:c r="G45" s="0" t="s">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="H45" s="0">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I45" s="0">
+        <x:v>120</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" spans="1:9">
+      <x:c r="A46" s="0">
+        <x:v>1029</x:v>
+      </x:c>
+      <x:c r="B46" s="0" t="s">
+        <x:v>79</x:v>
+      </x:c>
+      <x:c r="C46" s="0" t="s">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="D46" s="0" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="E46" s="0" t="s">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="F46" s="0" t="s">
+        <x:v>81</x:v>
+      </x:c>
+      <x:c r="G46" s="0" t="s">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="H46" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I46" s="0">
+        <x:v>90</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" spans="1:9">
+      <x:c r="A47" s="0">
+        <x:v>1029</x:v>
+      </x:c>
+      <x:c r="B47" s="0" t="s">
+        <x:v>79</x:v>
+      </x:c>
+      <x:c r="C47" s="0" t="s">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="D47" s="0" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="E47" s="0" t="s">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="F47" s="0" t="s">
+        <x:v>81</x:v>
+      </x:c>
+      <x:c r="G47" s="0" t="s">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="H47" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I47" s="0">
+        <x:v>90</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" spans="1:9">
+      <x:c r="A48" s="0">
+        <x:v>1030</x:v>
+      </x:c>
+      <x:c r="B48" s="0" t="s">
+        <x:v>82</x:v>
+      </x:c>
+      <x:c r="C48" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="D48" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E48" s="0" t="s">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="F48" s="0" t="s">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="G48" s="0" t="s">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="H48" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I48" s="0">
+        <x:v>150</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" spans="1:9">
+      <x:c r="A49" s="0">
+        <x:v>1030</x:v>
+      </x:c>
+      <x:c r="B49" s="0" t="s">
+        <x:v>82</x:v>
+      </x:c>
+      <x:c r="C49" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="D49" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E49" s="0" t="s">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="F49" s="0" t="s">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="G49" s="0" t="s">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="H49" s="0">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I49" s="0">
+        <x:v>150</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>

</xml_diff>

<commit_message>
feat: modern city dropdown + fix featured card strip + fix footer icons centering
- Replace radio button city list with searchable custom dropdown in checkout
- Add live search filter, keyboard navigation, price badges in dropdown
- Fix featured swiper card pink/purple strip: use fixed height, remove gradient bg
- Fix footer social icons: force center alignment on mobile with media query
- Fix Twilio: add credentials to appsettings.json, add null validation
- Change WhatsAppNotificationService from Singleton to Scoped
</commit_message>
<xml_diff>
--- a/Orkideya/wwwroot/orders.xlsx
+++ b/Orkideya/wwwroot/orders.xlsx
@@ -276,6 +276,12 @@
   </x:si>
   <x:si>
     <x:t>2026-02-26 03:46</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ضواحي طرابلس</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-03-07 06:57</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -2054,6 +2060,64 @@
         <x:v>150</x:v>
       </x:c>
     </x:row>
+    <x:row r="50" spans="1:9">
+      <x:c r="A50" s="0">
+        <x:v>1031</x:v>
+      </x:c>
+      <x:c r="B50" s="0" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="C50" s="0" t="s">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="D50" s="0" t="s">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="E50" s="0" t="s">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="F50" s="0" t="s">
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="G50" s="0" t="s">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="H50" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I50" s="0">
+        <x:v>95</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" spans="1:9">
+      <x:c r="A51" s="0">
+        <x:v>1031</x:v>
+      </x:c>
+      <x:c r="B51" s="0" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="C51" s="0" t="s">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="D51" s="0" t="s">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="E51" s="0" t="s">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="F51" s="0" t="s">
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="G51" s="0" t="s">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="H51" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I51" s="0">
+        <x:v>95</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>

</xml_diff>

<commit_message>
fix: featured swiper card - match all-products card style exactly
</commit_message>
<xml_diff>
--- a/Orkideya/wwwroot/orders.xlsx
+++ b/Orkideya/wwwroot/orders.xlsx
@@ -282,6 +282,12 @@
   </x:si>
   <x:si>
     <x:t>2026-03-07 06:57</x:t>
+  </x:si>
+  <x:si>
+    <x:t>مرزق</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-03-07 07:13</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -2118,6 +2124,64 @@
         <x:v>95</x:v>
       </x:c>
     </x:row>
+    <x:row r="52" spans="1:9">
+      <x:c r="A52" s="0">
+        <x:v>1032</x:v>
+      </x:c>
+      <x:c r="B52" s="0" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="C52" s="0" t="s">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="D52" s="0" t="s">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="E52" s="0" t="s">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="F52" s="0" t="s">
+        <x:v>88</x:v>
+      </x:c>
+      <x:c r="G52" s="0" t="s">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="H52" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I52" s="0">
+        <x:v>125</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" spans="1:9">
+      <x:c r="A53" s="0">
+        <x:v>1032</x:v>
+      </x:c>
+      <x:c r="B53" s="0" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="C53" s="0" t="s">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="D53" s="0" t="s">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="E53" s="0" t="s">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="F53" s="0" t="s">
+        <x:v>88</x:v>
+      </x:c>
+      <x:c r="G53" s="0" t="s">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="H53" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I53" s="0">
+        <x:v>125</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>

</xml_diff>

<commit_message>
fix: center footer badges on mobile
</commit_message>
<xml_diff>
--- a/Orkideya/wwwroot/orders.xlsx
+++ b/Orkideya/wwwroot/orders.xlsx
@@ -288,6 +288,12 @@
   </x:si>
   <x:si>
     <x:t>2026-03-07 07:13</x:t>
+  </x:si>
+  <x:si>
+    <x:t>سرت</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-03-07 07:32</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -2182,6 +2188,64 @@
         <x:v>125</x:v>
       </x:c>
     </x:row>
+    <x:row r="54" spans="1:9">
+      <x:c r="A54" s="0">
+        <x:v>1033</x:v>
+      </x:c>
+      <x:c r="B54" s="0" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="C54" s="0" t="s">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="D54" s="0" t="s">
+        <x:v>89</x:v>
+      </x:c>
+      <x:c r="E54" s="0" t="s">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="F54" s="0" t="s">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="G54" s="0" t="s">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="H54" s="0">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="I54" s="0">
+        <x:v>145</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" spans="1:9">
+      <x:c r="A55" s="0">
+        <x:v>1033</x:v>
+      </x:c>
+      <x:c r="B55" s="0" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="C55" s="0" t="s">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="D55" s="0" t="s">
+        <x:v>89</x:v>
+      </x:c>
+      <x:c r="E55" s="0" t="s">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="F55" s="0" t="s">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="G55" s="0" t="s">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="H55" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I55" s="0">
+        <x:v>145</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>

</xml_diff>